<commit_message>
I - #22 - fix asvs
</commit_message>
<xml_diff>
--- a/Derivables/Phase2/ASVS_5.0_Tracker_Kryptos.xlsx
+++ b/Derivables/Phase2/ASVS_5.0_Tracker_Kryptos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filipa/Documents/mestrado/desofs/desofs2026_thu_ffs_2/Derivables/Phase2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{831EDDA6-72B9-6146-A19D-66EDD061DD9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B669C1C-8BBD-D24A-AD74-4BB36EF31707}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17320" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3972,6 +3972,15 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3995,15 +4004,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4458,7 +4458,7 @@
                   <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>0.625</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -5343,46 +5343,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="36" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
-      <c r="L1" s="34"/>
-      <c r="M1" s="34"/>
-      <c r="N1" s="34"/>
-      <c r="O1" s="34"/>
-      <c r="P1" s="34"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+      <c r="P1" s="37"/>
     </row>
     <row r="2" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="36"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
-      <c r="M2" s="34"/>
-      <c r="N2" s="34"/>
-      <c r="O2" s="34"/>
-      <c r="P2" s="34"/>
+      <c r="A2" s="39"/>
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
+      <c r="L2" s="37"/>
+      <c r="M2" s="37"/>
+      <c r="N2" s="37"/>
+      <c r="O2" s="37"/>
+      <c r="P2" s="37"/>
     </row>
     <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="35"/>
-      <c r="B3" s="34"/>
+      <c r="A3" s="38"/>
+      <c r="B3" s="37"/>
       <c r="C3" s="1"/>
       <c r="E3" s="1"/>
       <c r="G3" s="1"/>
@@ -5619,7 +5619,7 @@
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="L9" s="44">
+      <c r="L9" s="34">
         <f>COUNTIF('V4 - API and Web Service'!$F$2:$F$21,"Compliant")</f>
         <v>9</v>
       </c>
@@ -5668,7 +5668,7 @@
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
-      <c r="L10" s="45">
+      <c r="L10" s="35">
         <f>COUNTIF('V5 - File Handling'!$F$2:$F$18,"Compliant")</f>
         <v>12</v>
       </c>
@@ -5717,7 +5717,7 @@
         <f t="shared" si="2"/>
         <v>0.58333333333333337</v>
       </c>
-      <c r="L11" s="44">
+      <c r="L11" s="34">
         <f>COUNTIF('V6 - Authentication'!$F$2:$F$56,"Compliant")</f>
         <v>30</v>
       </c>
@@ -5766,7 +5766,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L12" s="45">
+      <c r="L12" s="35">
         <f>COUNTIF('V7 - Session Management'!$F$2:$F$26,"Compliant")</f>
         <v>12</v>
       </c>
@@ -5815,7 +5815,7 @@
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="L13" s="44">
+      <c r="L13" s="34">
         <f>COUNTIF('V8 - Authorization'!$F$2:$F$18,"Compliant")</f>
         <v>8</v>
       </c>
@@ -5864,7 +5864,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="L14" s="45">
+      <c r="L14" s="35">
         <f>COUNTIF('V9 - Self-contained Tokens'!$F$2:$F$10,"Compliant")</f>
         <v>6</v>
       </c>
@@ -5913,7 +5913,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L15" s="44">
+      <c r="L15" s="34">
         <f>COUNTIF('V10 - OAuth and OIDC'!$F$2:$F$44,"Compliant")</f>
         <v>5</v>
       </c>
@@ -5962,7 +5962,7 @@
         <f t="shared" si="2"/>
         <v>0.8</v>
       </c>
-      <c r="L16" s="45">
+      <c r="L16" s="35">
         <f>COUNTIF('V11 - Cryptography'!$F$2:$F$32,"Compliant")</f>
         <v>22</v>
       </c>
@@ -6011,7 +6011,7 @@
         <f t="shared" si="2"/>
         <v>0.66666666666666663</v>
       </c>
-      <c r="L17" s="44">
+      <c r="L17" s="34">
         <f>COUNTIF('V12 - Secure Communication'!$F$2:$F$16,"Compliant")</f>
         <v>10</v>
       </c>
@@ -6060,7 +6060,7 @@
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="L18" s="45">
+      <c r="L18" s="35">
         <f>COUNTIF('V13 - Configuration'!$F$2:$F$26,"Compliant")</f>
         <v>21</v>
       </c>
@@ -6109,7 +6109,7 @@
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="L19" s="44">
+      <c r="L19" s="34">
         <f>COUNTIF('V14 - Data Protection'!$F$2:$F$17,"Compliant")</f>
         <v>8</v>
       </c>
@@ -6158,7 +6158,7 @@
         <f t="shared" si="2"/>
         <v>0.375</v>
       </c>
-      <c r="L20" s="45">
+      <c r="L20" s="35">
         <f>COUNTIF('V15 - Secure Coding and Archite'!$F$2:$F$26,"Compliant")</f>
         <v>11</v>
       </c>
@@ -6181,7 +6181,7 @@
         <f>COUNTIFS('V16 - Security Logging and Erro'!E3:E23,"Compliant",'V16 - Security Logging and Erro'!F3:F23,1)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="43" t="str">
+      <c r="E21" s="33" t="str">
         <f>IF(C21=0,"",D21/C21)</f>
         <v/>
       </c>
@@ -6189,25 +6189,25 @@
         <v>16</v>
       </c>
       <c r="G21" s="4">
-        <f>COUNTIFS('V16 - Security Logging and Erro'!H3:H23,"Compliant",'V16 - Security Logging and Erro'!I3:I23,2)</f>
-        <v>0</v>
+        <f>COUNTIFS('V16 - Security Logging and Erro'!F3:F23,"Compliant",'V16 - Security Logging and Erro'!E3:E23,2)</f>
+        <v>10</v>
       </c>
       <c r="H21" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.625</v>
       </c>
       <c r="I21" s="7">
         <v>1</v>
       </c>
       <c r="J21" s="4">
-        <f>COUNTIFS('V16 - Security Logging and Erro'!K3:K23,"Compliant",'V16 - Security Logging and Erro'!L3:L23,3)</f>
+        <f>COUNTIFS('V16 - Security Logging and Erro'!F3:F23,"Compliant",'V16 - Security Logging and Erro'!E3:E23,3)</f>
         <v>0</v>
       </c>
       <c r="K21" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L21" s="44">
+      <c r="L21" s="34">
         <f>COUNTIF('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant")</f>
         <v>10</v>
       </c>
@@ -6230,7 +6230,7 @@
         <f>COUNTIFS('V17 - WebRTC'!E3:E16,"Compliant",'V17 - WebRTC'!F3:F16,1)</f>
         <v>0</v>
       </c>
-      <c r="E22" s="43" t="str">
+      <c r="E22" s="33" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -6238,7 +6238,7 @@
         <v>7</v>
       </c>
       <c r="G22" s="4">
-        <f>COUNTIFS('V17 - WebRTC'!H3:H16,"Compliant",'V17 - WebRTC'!I3:I16,2)</f>
+        <f>COUNTIFS('V17 - WebRTC'!F3:F16,"Compliant",'V17 - WebRTC'!E3:E16,2)</f>
         <v>0</v>
       </c>
       <c r="H22" s="5">
@@ -6249,14 +6249,14 @@
         <v>5</v>
       </c>
       <c r="J22" s="4">
-        <f>COUNTIFS('V17 - WebRTC'!K3:K16,"Compliant",'V17 - WebRTC'!L3:L16,3)</f>
+        <f>COUNTIFS('V17 - WebRTC'!F3:F16,"Compliant",'V17 - WebRTC'!E3:E16,3)</f>
         <v>0</v>
       </c>
       <c r="K22" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L22" s="45">
+      <c r="L22" s="35">
         <f>COUNTIF('V17 - WebRTC'!$F$2:$F$16,"Compliant")</f>
         <v>0</v>
       </c>
@@ -6289,11 +6289,11 @@
       </c>
       <c r="G23" s="9">
         <f>SUM(G6:G22)</f>
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H23" s="10">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>0.54070838861860526</v>
+        <v>0.57747309450095829</v>
       </c>
       <c r="I23" s="9">
         <f>SUM(I6:I22)</f>
@@ -9539,11 +9539,11 @@
         <v>1013</v>
       </c>
       <c r="H3" s="15"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="34"/>
-      <c r="K3" s="34"/>
-      <c r="L3" s="34"/>
-      <c r="M3" s="34"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="37"/>
+      <c r="K3" s="37"/>
+      <c r="L3" s="37"/>
+      <c r="M3" s="37"/>
     </row>
     <row r="4" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="18" t="s">
@@ -9568,11 +9568,11 @@
         <v>1016</v>
       </c>
       <c r="H4" s="20"/>
-      <c r="I4" s="38"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="34"/>
-      <c r="M4" s="34"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="37"/>
+      <c r="K4" s="37"/>
+      <c r="L4" s="37"/>
+      <c r="M4" s="37"/>
     </row>
     <row r="5" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
@@ -9611,11 +9611,11 @@
         <v>1021</v>
       </c>
       <c r="H6" s="15"/>
-      <c r="I6" s="37"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="34"/>
-      <c r="M6" s="34"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="37"/>
+      <c r="K6" s="37"/>
+      <c r="L6" s="37"/>
+      <c r="M6" s="37"/>
     </row>
     <row r="7" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="18" t="s">
@@ -9638,11 +9638,11 @@
       </c>
       <c r="G7" s="30"/>
       <c r="H7" s="20"/>
-      <c r="I7" s="39"/>
-      <c r="J7" s="34"/>
-      <c r="K7" s="34"/>
-      <c r="L7" s="34"/>
-      <c r="M7" s="34"/>
+      <c r="I7" s="42"/>
+      <c r="J7" s="37"/>
+      <c r="K7" s="37"/>
+      <c r="L7" s="37"/>
+      <c r="M7" s="37"/>
     </row>
     <row r="8" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="13" t="s">
@@ -9667,11 +9667,11 @@
         <v>1026</v>
       </c>
       <c r="H8" s="15"/>
-      <c r="I8" s="39"/>
-      <c r="J8" s="34"/>
-      <c r="K8" s="34"/>
-      <c r="L8" s="34"/>
-      <c r="M8" s="34"/>
+      <c r="I8" s="42"/>
+      <c r="J8" s="37"/>
+      <c r="K8" s="37"/>
+      <c r="L8" s="37"/>
+      <c r="M8" s="37"/>
     </row>
     <row r="9" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="18" t="s">
@@ -9696,11 +9696,11 @@
         <v>1029</v>
       </c>
       <c r="H9" s="20"/>
-      <c r="I9" s="39"/>
-      <c r="J9" s="34"/>
-      <c r="K9" s="34"/>
-      <c r="L9" s="34"/>
-      <c r="M9" s="34"/>
+      <c r="I9" s="42"/>
+      <c r="J9" s="37"/>
+      <c r="K9" s="37"/>
+      <c r="L9" s="37"/>
+      <c r="M9" s="37"/>
     </row>
     <row r="10" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="13" t="s">
@@ -9769,11 +9769,11 @@
         <v>1036</v>
       </c>
       <c r="H12" s="15"/>
-      <c r="I12" s="41"/>
-      <c r="J12" s="34"/>
-      <c r="K12" s="34"/>
-      <c r="L12" s="34"/>
-      <c r="M12" s="34"/>
+      <c r="I12" s="44"/>
+      <c r="J12" s="37"/>
+      <c r="K12" s="37"/>
+      <c r="L12" s="37"/>
+      <c r="M12" s="37"/>
     </row>
     <row r="13" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="18" t="s">
@@ -9798,11 +9798,11 @@
         <v>1039</v>
       </c>
       <c r="H13" s="20"/>
-      <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
-      <c r="K13" s="34"/>
-      <c r="L13" s="34"/>
-      <c r="M13" s="34"/>
+      <c r="I13" s="40"/>
+      <c r="J13" s="37"/>
+      <c r="K13" s="37"/>
+      <c r="L13" s="37"/>
+      <c r="M13" s="37"/>
     </row>
     <row r="14" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
@@ -9865,11 +9865,11 @@
       <c r="H16" s="20" t="s">
         <v>1047</v>
       </c>
-      <c r="I16" s="40"/>
-      <c r="J16" s="34"/>
-      <c r="K16" s="34"/>
-      <c r="L16" s="34"/>
-      <c r="M16" s="34"/>
+      <c r="I16" s="43"/>
+      <c r="J16" s="37"/>
+      <c r="K16" s="37"/>
+      <c r="L16" s="37"/>
+      <c r="M16" s="37"/>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13" t="s">
@@ -10004,10 +10004,10 @@
         <v>1054</v>
       </c>
       <c r="H3" s="15"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="34"/>
-      <c r="K3" s="34"/>
-      <c r="L3" s="34"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="37"/>
+      <c r="K3" s="37"/>
+      <c r="L3" s="37"/>
     </row>
     <row r="4" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="18" t="s">
@@ -10034,10 +10034,10 @@
       <c r="H4" s="20" t="s">
         <v>1058</v>
       </c>
-      <c r="I4" s="38"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="34"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="37"/>
+      <c r="K4" s="37"/>
+      <c r="L4" s="37"/>
     </row>
     <row r="5" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="13" t="s">
@@ -10064,10 +10064,10 @@
       <c r="H5" s="15" t="s">
         <v>1062</v>
       </c>
-      <c r="I5" s="38"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
     </row>
     <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="18" t="s">
@@ -10092,10 +10092,10 @@
         <v>1065</v>
       </c>
       <c r="H6" s="20"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="34"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="37"/>
+      <c r="K6" s="37"/>
+      <c r="L6" s="37"/>
     </row>
     <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="13" t="s">
@@ -10120,10 +10120,10 @@
         <v>1068</v>
       </c>
       <c r="H7" s="15"/>
-      <c r="I7" s="38"/>
-      <c r="J7" s="34"/>
-      <c r="K7" s="34"/>
-      <c r="L7" s="34"/>
+      <c r="I7" s="41"/>
+      <c r="J7" s="37"/>
+      <c r="K7" s="37"/>
+      <c r="L7" s="37"/>
     </row>
     <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
@@ -10164,10 +10164,10 @@
       <c r="H9" s="15" t="s">
         <v>1074</v>
       </c>
-      <c r="I9" s="37"/>
-      <c r="J9" s="34"/>
-      <c r="K9" s="34"/>
-      <c r="L9" s="34"/>
+      <c r="I9" s="40"/>
+      <c r="J9" s="37"/>
+      <c r="K9" s="37"/>
+      <c r="L9" s="37"/>
     </row>
     <row r="10" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="18" t="s">
@@ -10190,10 +10190,10 @@
       </c>
       <c r="G10" s="20"/>
       <c r="H10" s="20"/>
-      <c r="I10" s="38"/>
-      <c r="J10" s="34"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="34"/>
+      <c r="I10" s="41"/>
+      <c r="J10" s="37"/>
+      <c r="K10" s="37"/>
+      <c r="L10" s="37"/>
     </row>
     <row r="11" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="13" t="s">
@@ -10220,10 +10220,10 @@
       <c r="H11" s="15" t="s">
         <v>1080</v>
       </c>
-      <c r="I11" s="38"/>
-      <c r="J11" s="34"/>
-      <c r="K11" s="34"/>
-      <c r="L11" s="34"/>
+      <c r="I11" s="41"/>
+      <c r="J11" s="37"/>
+      <c r="K11" s="37"/>
+      <c r="L11" s="37"/>
     </row>
     <row r="12" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="18" t="s">
@@ -10308,10 +10308,10 @@
       <c r="H15" s="15" t="s">
         <v>1090</v>
       </c>
-      <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
-      <c r="K15" s="34"/>
-      <c r="L15" s="34"/>
+      <c r="I15" s="40"/>
+      <c r="J15" s="37"/>
+      <c r="K15" s="37"/>
+      <c r="L15" s="37"/>
     </row>
     <row r="16" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="18" t="s">
@@ -10360,10 +10360,10 @@
       <c r="H17" s="23" t="s">
         <v>1096</v>
       </c>
-      <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
-      <c r="K17" s="34"/>
-      <c r="L17" s="34"/>
+      <c r="I17" s="40"/>
+      <c r="J17" s="37"/>
+      <c r="K17" s="37"/>
+      <c r="L17" s="37"/>
     </row>
     <row r="18" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="18" t="s">
@@ -10412,10 +10412,10 @@
       <c r="H19" s="15" t="s">
         <v>1102</v>
       </c>
-      <c r="I19" s="42"/>
-      <c r="J19" s="34"/>
-      <c r="K19" s="34"/>
-      <c r="L19" s="34"/>
+      <c r="I19" s="45"/>
+      <c r="J19" s="37"/>
+      <c r="K19" s="37"/>
+      <c r="L19" s="37"/>
     </row>
     <row r="20" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="18" t="s">
@@ -10496,10 +10496,10 @@
       </c>
       <c r="G23" s="15"/>
       <c r="H23" s="15"/>
-      <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
-      <c r="K23" s="34"/>
-      <c r="L23" s="34"/>
+      <c r="I23" s="40"/>
+      <c r="J23" s="37"/>
+      <c r="K23" s="37"/>
+      <c r="L23" s="37"/>
     </row>
     <row r="24" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="18" t="s">
@@ -10526,10 +10526,10 @@
       <c r="H24" s="20" t="s">
         <v>1114</v>
       </c>
-      <c r="I24" s="38"/>
-      <c r="J24" s="34"/>
-      <c r="K24" s="34"/>
-      <c r="L24" s="34"/>
+      <c r="I24" s="41"/>
+      <c r="J24" s="37"/>
+      <c r="K24" s="37"/>
+      <c r="L24" s="37"/>
     </row>
     <row r="25" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="13" t="s">
@@ -10552,10 +10552,10 @@
       </c>
       <c r="G25" s="15"/>
       <c r="H25" s="15"/>
-      <c r="I25" s="38"/>
-      <c r="J25" s="34"/>
-      <c r="K25" s="34"/>
-      <c r="L25" s="34"/>
+      <c r="I25" s="41"/>
+      <c r="J25" s="37"/>
+      <c r="K25" s="37"/>
+      <c r="L25" s="37"/>
     </row>
     <row r="26" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="18" t="s">
@@ -10578,10 +10578,10 @@
       </c>
       <c r="G26" s="20"/>
       <c r="H26" s="20"/>
-      <c r="I26" s="38"/>
-      <c r="J26" s="34"/>
-      <c r="K26" s="34"/>
-      <c r="L26" s="34"/>
+      <c r="I26" s="41"/>
+      <c r="J26" s="37"/>
+      <c r="K26" s="37"/>
+      <c r="L26" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -10668,10 +10668,10 @@
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
       <c r="H2" s="12"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
+      <c r="L2" s="37"/>
     </row>
     <row r="3" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="s">
@@ -10698,10 +10698,10 @@
       <c r="H3" s="15" t="s">
         <v>1124</v>
       </c>
-      <c r="I3" s="42"/>
-      <c r="J3" s="34"/>
-      <c r="K3" s="34"/>
-      <c r="L3" s="34"/>
+      <c r="I3" s="45"/>
+      <c r="J3" s="37"/>
+      <c r="K3" s="37"/>
+      <c r="L3" s="37"/>
     </row>
     <row r="4" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
@@ -10740,10 +10740,10 @@
         <v>1129</v>
       </c>
       <c r="H5" s="15"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
+      <c r="I5" s="45"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
     </row>
     <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="18" t="s">
@@ -10768,10 +10768,10 @@
         <v>1132</v>
       </c>
       <c r="H6" s="20"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="34"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="37"/>
+      <c r="K6" s="37"/>
+      <c r="L6" s="37"/>
     </row>
     <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="13" t="s">
@@ -10876,10 +10876,10 @@
         <v>1143</v>
       </c>
       <c r="H11" s="15"/>
-      <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
-      <c r="K11" s="34"/>
-      <c r="L11" s="34"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="37"/>
+      <c r="K11" s="37"/>
+      <c r="L11" s="37"/>
     </row>
     <row r="12" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="18" t="s">
@@ -10904,10 +10904,10 @@
         <v>1146</v>
       </c>
       <c r="H12" s="20"/>
-      <c r="I12" s="38"/>
-      <c r="J12" s="34"/>
-      <c r="K12" s="34"/>
-      <c r="L12" s="34"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="37"/>
+      <c r="K12" s="37"/>
+      <c r="L12" s="37"/>
     </row>
     <row r="13" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="13" t="s">
@@ -10932,10 +10932,10 @@
         <v>1149</v>
       </c>
       <c r="H13" s="15"/>
-      <c r="I13" s="38"/>
-      <c r="J13" s="34"/>
-      <c r="K13" s="34"/>
-      <c r="L13" s="34"/>
+      <c r="I13" s="41"/>
+      <c r="J13" s="37"/>
+      <c r="K13" s="37"/>
+      <c r="L13" s="37"/>
     </row>
     <row r="14" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="18" t="s">
@@ -10960,10 +10960,10 @@
         <v>1152</v>
       </c>
       <c r="H14" s="20"/>
-      <c r="I14" s="38"/>
-      <c r="J14" s="34"/>
-      <c r="K14" s="34"/>
-      <c r="L14" s="34"/>
+      <c r="I14" s="41"/>
+      <c r="J14" s="37"/>
+      <c r="K14" s="37"/>
+      <c r="L14" s="37"/>
     </row>
     <row r="15" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
@@ -11026,10 +11026,10 @@
       <c r="H17" s="20" t="s">
         <v>1160</v>
       </c>
-      <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
-      <c r="K17" s="34"/>
-      <c r="L17" s="34"/>
+      <c r="I17" s="40"/>
+      <c r="J17" s="37"/>
+      <c r="K17" s="37"/>
+      <c r="L17" s="37"/>
     </row>
     <row r="18" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="13" t="s">
@@ -11054,10 +11054,10 @@
         <v>1163</v>
       </c>
       <c r="H18" s="15"/>
-      <c r="I18" s="38"/>
-      <c r="J18" s="34"/>
-      <c r="K18" s="34"/>
-      <c r="L18" s="34"/>
+      <c r="I18" s="41"/>
+      <c r="J18" s="37"/>
+      <c r="K18" s="37"/>
+      <c r="L18" s="37"/>
     </row>
     <row r="19" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="12" t="s">
@@ -11098,10 +11098,10 @@
       <c r="H20" s="15" t="s">
         <v>1169</v>
       </c>
-      <c r="I20" s="42"/>
-      <c r="J20" s="34"/>
-      <c r="K20" s="34"/>
-      <c r="L20" s="34"/>
+      <c r="I20" s="45"/>
+      <c r="J20" s="37"/>
+      <c r="K20" s="37"/>
+      <c r="L20" s="37"/>
     </row>
     <row r="21" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="18" t="s">

</xml_diff>